<commit_message>
Normalize calendar xlsx for Google Sheets conversion
Rebuild the workbook with the layout that Drive's converter accepts
(9-column grid, uniform fills), keeping the X-first sell-to-projects
content unchanged.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HeCjF7fsjCUn5ySBJ1uikn
</commit_message>
<xml_diff>
--- a/marketing/permissionless_campaigns_calendar.xlsx
+++ b/marketing/permissionless_campaigns_calendar.xlsx
@@ -47,7 +47,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -76,27 +76,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CFE2F3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FCE5CD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EAD1DC"/>
       </patternFill>
     </fill>
   </fills>
@@ -126,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -147,16 +132,7 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -530,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -541,6 +517,7 @@
     <col width="27" customWidth="1" min="6" max="6"/>
     <col width="27" customWidth="1" min="7" max="7"/>
     <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -591,11 +568,12 @@
           <t>Sunday</t>
         </is>
       </c>
+      <c r="I2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Week of Aug 03 – Aug 09, 2026 (NARRATIVE + TEASER)</t>
+          <t>Week of Aug 03 - Aug 09, 2026 (NARRATIVE + TEASER)</t>
         </is>
       </c>
       <c r="B3" s="4" t="n"/>
@@ -605,8 +583,9 @@
       <c r="F3" s="4" t="n"/>
       <c r="G3" s="4" t="n"/>
       <c r="H3" s="4" t="n"/>
-    </row>
-    <row r="4" ht="16" customHeight="1">
+      <c r="I3" s="4" t="n"/>
+    </row>
+    <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Action Release</t>
@@ -619,8 +598,9 @@
       <c r="F4" s="6" t="inlineStr"/>
       <c r="G4" s="6" t="inlineStr"/>
       <c r="H4" s="6" t="inlineStr"/>
-    </row>
-    <row r="5" ht="50" customHeight="1">
+      <c r="I4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5" ht="55" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Video</t>
@@ -632,38 +612,40 @@
       <c r="E5" s="6" t="inlineStr"/>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Demo teaser — 15s cutdown of the Demo Video</t>
+          <t>Demo teaser - 15s cutdown of the Demo Video</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr"/>
       <c r="H5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6" ht="50" customHeight="1">
+      <c r="I5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6" ht="55" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>X — Announcement</t>
+          <t>X - Announcement</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr"/>
       <c r="C6" s="6" t="inlineStr"/>
       <c r="D6" s="6" t="inlineStr"/>
       <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Something permissionless is coming (TEASER POST)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>Countdown — launch date reveal (POST)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Countdown - launch date reveal (POST)</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>X — Sell to Projects</t>
+          <t>X - Sell to Projects</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr"/>
@@ -673,17 +655,18 @@
       <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="6" t="inlineStr"/>
       <c r="H7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8" ht="50" customHeight="1">
+      <c r="I7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="55" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Article</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr"/>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>The Protocol Narrative — campaigns without gatekeepers (ARTICLE)</t>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>The Protocol Narrative - campaigns without gatekeepers (ARTICLE)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr"/>
@@ -691,8 +674,9 @@
       <c r="F8" s="6" t="inlineStr"/>
       <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9" ht="16" customHeight="1">
+      <c r="I8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>X Space / Live</t>
@@ -705,8 +689,9 @@
       <c r="F9" s="6" t="inlineStr"/>
       <c r="G9" s="6" t="inlineStr"/>
       <c r="H9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="50" customHeight="1">
+      <c r="I9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10" ht="55" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Creators &amp; Communities</t>
@@ -727,8 +712,9 @@
       <c r="F10" s="6" t="inlineStr"/>
       <c r="G10" s="6" t="inlineStr"/>
       <c r="H10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11" ht="50" customHeight="1">
+      <c r="I10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11" ht="55" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>BD / Projects</t>
@@ -749,8 +735,9 @@
       <c r="F11" s="6" t="inlineStr"/>
       <c r="G11" s="6" t="inlineStr"/>
       <c r="H11" s="6" t="inlineStr"/>
-    </row>
-    <row r="12" ht="16" customHeight="1">
+      <c r="I11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>PR</t>
@@ -763,8 +750,9 @@
       <c r="F12" s="6" t="inlineStr"/>
       <c r="G12" s="6" t="inlineStr"/>
       <c r="H12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13" ht="16" customHeight="1">
+      <c r="I12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Mailing</t>
@@ -777,8 +765,9 @@
       <c r="F13" s="6" t="inlineStr"/>
       <c r="G13" s="6" t="inlineStr"/>
       <c r="H13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14" ht="16" customHeight="1">
+      <c r="I13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>KOL</t>
@@ -791,11 +780,12 @@
       <c r="F14" s="6" t="inlineStr"/>
       <c r="G14" s="6" t="inlineStr"/>
       <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="4" t="inlineStr"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Week of Aug 10 – Aug 16, 2026 (LAUNCH)</t>
+          <t>Week of Aug 10 - Aug 16, 2026 (LAUNCH)</t>
         </is>
       </c>
       <c r="B16" s="4" t="n"/>
@@ -805,14 +795,15 @@
       <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="n"/>
       <c r="H16" s="4" t="n"/>
-    </row>
-    <row r="17" ht="50" customHeight="1">
+      <c r="I16" s="4" t="n"/>
+    </row>
+    <row r="17" ht="55" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Action Release</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>PERMISSIONLESS CAMPAIGNS LIVE</t>
         </is>
@@ -823,8 +814,9 @@
       <c r="F17" s="6" t="inlineStr"/>
       <c r="G17" s="6" t="inlineStr"/>
       <c r="H17" s="6" t="inlineStr"/>
-    </row>
-    <row r="18" ht="50" customHeight="1">
+      <c r="I17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18" ht="55" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Video</t>
@@ -832,7 +824,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>DEMO VIDEO — hero piece: create &amp; launch a campaign end-to-end</t>
+          <t>DEMO VIDEO - hero piece: create &amp; launch a campaign end-to-end</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr"/>
@@ -841,14 +833,15 @@
       <c r="F18" s="6" t="inlineStr"/>
       <c r="G18" s="6" t="inlineStr"/>
       <c r="H18" s="6" t="inlineStr"/>
-    </row>
-    <row r="19" ht="50" customHeight="1">
+      <c r="I18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19" ht="55" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>X — Announcement</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
+          <t>X - Announcement</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Launch thread + Demo Video (pinned)</t>
         </is>
@@ -859,43 +852,45 @@
       <c r="F19" s="6" t="inlineStr"/>
       <c r="G19" s="6" t="inlineStr"/>
       <c r="H19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20" ht="50" customHeight="1">
+      <c r="I19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20" ht="55" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>X — Sell to Projects</t>
+          <t>X - Sell to Projects</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr"/>
       <c r="C20" s="6" t="inlineStr"/>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>Verified Campaigns — what 1,500$ gets your project: protocol visibility, Rally marketing pack, elite creators &amp; ambassadors (THREAD + ONE-PAGER)</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>Network Campaigns — permissionless, rewards in USDC | RLPs (THREAD + Verified vs Network VISUAL)</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>CALL FOR PROJECTS — launching soon? Run your launch as a Network Campaign (POST + form)</t>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Verified Campaigns - what 1,500$ gets your project: protocol visibility, Rally marketing pack, elite creators &amp; ambassadors (THREAD + ONE-PAGER)</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Network Campaigns - permissionless, rewards in USDC | RLPs (THREAD + Verified vs Network VISUAL)</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>CALL FOR PROJECTS - launching soon? Run your launch as a Network Campaign (POST + form)</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr"/>
       <c r="H20" s="6" t="inlineStr"/>
-    </row>
-    <row r="21" ht="50" customHeight="1">
+      <c r="I20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21" ht="55" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Article</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr"/>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>Permissionless Campaigns: how it works — pay in RLPs | USDC (ARTICLE)</t>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Permissionless Campaigns: how it works - pay in RLPs | USDC (ARTICLE)</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr"/>
@@ -903,8 +898,9 @@
       <c r="F21" s="6" t="inlineStr"/>
       <c r="G21" s="6" t="inlineStr"/>
       <c r="H21" s="6" t="inlineStr"/>
-    </row>
-    <row r="22" ht="16" customHeight="1">
+      <c r="I21" s="4" t="inlineStr"/>
+    </row>
+    <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t>X Space / Live</t>
@@ -917,8 +913,9 @@
       <c r="F22" s="6" t="inlineStr"/>
       <c r="G22" s="6" t="inlineStr"/>
       <c r="H22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23" ht="50" customHeight="1">
+      <c r="I22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23" ht="55" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Creators &amp; Communities</t>
@@ -926,7 +923,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Coordinated push — communities &amp; creators RT/QT the launch simultaneously</t>
+          <t>Coordinated push - communities &amp; creators RT/QT the launch simultaneously</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr"/>
@@ -939,8 +936,9 @@
       </c>
       <c r="G23" s="6" t="inlineStr"/>
       <c r="H23" s="6" t="inlineStr"/>
-    </row>
-    <row r="24" ht="16" customHeight="1">
+      <c r="I23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
           <t>BD / Projects</t>
@@ -953,8 +951,9 @@
       <c r="F24" s="6" t="inlineStr"/>
       <c r="G24" s="6" t="inlineStr"/>
       <c r="H24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25" ht="16" customHeight="1">
+      <c r="I24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>PR</t>
@@ -967,8 +966,9 @@
       <c r="F25" s="6" t="inlineStr"/>
       <c r="G25" s="6" t="inlineStr"/>
       <c r="H25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26" ht="50" customHeight="1">
+      <c r="I25" s="4" t="inlineStr"/>
+    </row>
+    <row r="26" ht="55" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Mailing</t>
@@ -989,8 +989,9 @@
       <c r="F26" s="6" t="inlineStr"/>
       <c r="G26" s="6" t="inlineStr"/>
       <c r="H26" s="6" t="inlineStr"/>
-    </row>
-    <row r="27" ht="50" customHeight="1">
+      <c r="I26" s="4" t="inlineStr"/>
+    </row>
+    <row r="27" ht="55" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>KOL</t>
@@ -1007,11 +1008,12 @@
       <c r="F27" s="6" t="inlineStr"/>
       <c r="G27" s="6" t="inlineStr"/>
       <c r="H27" s="6" t="inlineStr"/>
+      <c r="I27" s="4" t="inlineStr"/>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Week of Aug 17 – Aug 23, 2026 (SELL TO PROJECTS + CREATORS)</t>
+          <t>Week of Aug 17 - Aug 23, 2026 (SELL TO PROJECTS + CREATORS)</t>
         </is>
       </c>
       <c r="B29" s="4" t="n"/>
@@ -1021,8 +1023,9 @@
       <c r="F29" s="4" t="n"/>
       <c r="G29" s="4" t="n"/>
       <c r="H29" s="4" t="n"/>
-    </row>
-    <row r="30" ht="16" customHeight="1">
+      <c r="I29" s="4" t="n"/>
+    </row>
+    <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Action Release</t>
@@ -1035,8 +1038,9 @@
       <c r="F30" s="6" t="inlineStr"/>
       <c r="G30" s="6" t="inlineStr"/>
       <c r="H30" s="6" t="inlineStr"/>
-    </row>
-    <row r="31" ht="50" customHeight="1">
+      <c r="I30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31" ht="55" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Video</t>
@@ -1046,27 +1050,28 @@
       <c r="C31" s="6" t="inlineStr"/>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Creator video #1 — 'I launched a campaign, here's my experience'</t>
+          <t>Creator video #1 - 'I launched a campaign, here is my experience'</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr"/>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Demo cutdown #2 — project POV: 'your launch could look like this'</t>
+          <t>Demo cutdown #2 - project POV: 'your launch could look like this'</t>
         </is>
       </c>
       <c r="G31" s="6" t="inlineStr"/>
       <c r="H31" s="6" t="inlineStr"/>
-    </row>
-    <row r="32" ht="50" customHeight="1">
+      <c r="I31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32" ht="55" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>X — Announcement</t>
-        </is>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>First 10 Network Campaigns — spotlight (THREAD)</t>
+          <t>X - Announcement</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>First 10 Network Campaigns - spotlight (THREAD)</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr"/>
@@ -1075,17 +1080,18 @@
       <c r="F32" s="6" t="inlineStr"/>
       <c r="G32" s="6" t="inlineStr"/>
       <c r="H32" s="6" t="inlineStr"/>
-    </row>
-    <row r="33" ht="50" customHeight="1">
+      <c r="I32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33" ht="55" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>X — Sell to Projects</t>
+          <t>X - Sell to Projects</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr"/>
-      <c r="C33" s="11" t="inlineStr">
-        <is>
-          <t>Why your project should create a Network Campaign — 5 use cases (THREAD, links article)</t>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Why your project should create a Network Campaign - 5 use cases (THREAD, links article)</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr"/>
@@ -1093,30 +1099,32 @@
       <c r="F33" s="6" t="inlineStr"/>
       <c r="G33" s="6" t="inlineStr"/>
       <c r="H33" s="6" t="inlineStr"/>
-    </row>
-    <row r="34" ht="50" customHeight="1">
+      <c r="I33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34" ht="55" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
           <t>Article</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr"/>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>Why create a Network Campaign — 5 use cases (ARTICLE, sales-ready)</t>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Why create a Network Campaign - 5 use cases (ARTICLE, sales-ready)</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr"/>
-      <c r="E34" s="9" t="inlineStr">
-        <is>
-          <t>Viraliza tu Launch — playbook for projects (ARTICLE)</t>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Viraliza tu Launch - playbook for projects (ARTICLE)</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr"/>
       <c r="G34" s="6" t="inlineStr"/>
       <c r="H34" s="6" t="inlineStr"/>
-    </row>
-    <row r="35" ht="50" customHeight="1">
+      <c r="I34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35" ht="55" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
           <t>X Space / Live</t>
@@ -1126,19 +1134,20 @@
       <c r="C35" s="6" t="inlineStr"/>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Live demo for projects — launch a campaign in 10 minutes (X SPACE/VIDEO)</t>
+          <t>Live demo for projects - launch a campaign in 10 minutes (X SPACE/VIDEO)</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr"/>
       <c r="F35" s="6" t="inlineStr"/>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>X Space with communities &amp; creators — first campaigns debrief</t>
+          <t>X Space with communities &amp; creators - first campaigns debrief</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr"/>
-    </row>
-    <row r="36" ht="50" customHeight="1">
+      <c r="I35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36" ht="55" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
           <t>Creators &amp; Communities</t>
@@ -1155,8 +1164,9 @@
       <c r="F36" s="6" t="inlineStr"/>
       <c r="G36" s="6" t="inlineStr"/>
       <c r="H36" s="6" t="inlineStr"/>
-    </row>
-    <row r="37" ht="50" customHeight="1">
+      <c r="I36" s="4" t="inlineStr"/>
+    </row>
+    <row r="37" ht="55" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
           <t>BD / Projects</t>
@@ -1173,8 +1183,9 @@
       <c r="F37" s="6" t="inlineStr"/>
       <c r="G37" s="6" t="inlineStr"/>
       <c r="H37" s="6" t="inlineStr"/>
-    </row>
-    <row r="38" ht="16" customHeight="1">
+      <c r="I37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
           <t>PR</t>
@@ -1187,8 +1198,9 @@
       <c r="F38" s="6" t="inlineStr"/>
       <c r="G38" s="6" t="inlineStr"/>
       <c r="H38" s="6" t="inlineStr"/>
-    </row>
-    <row r="39" ht="50" customHeight="1">
+      <c r="I38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39" ht="55" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
         <is>
           <t>Mailing</t>
@@ -1205,8 +1217,9 @@
       <c r="F39" s="6" t="inlineStr"/>
       <c r="G39" s="6" t="inlineStr"/>
       <c r="H39" s="6" t="inlineStr"/>
-    </row>
-    <row r="40" ht="50" customHeight="1">
+      <c r="I39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40" ht="55" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
         <is>
           <t>KOL</t>
@@ -1223,11 +1236,12 @@
       <c r="F40" s="6" t="inlineStr"/>
       <c r="G40" s="6" t="inlineStr"/>
       <c r="H40" s="6" t="inlineStr"/>
+      <c r="I40" s="4" t="inlineStr"/>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Week of Aug 24 – Aug 30, 2026 (SOCIAL PROOF + PR)</t>
+          <t>Week of Aug 24 - Aug 30, 2026 (SOCIAL PROOF + PR)</t>
         </is>
       </c>
       <c r="B42" s="4" t="n"/>
@@ -1237,8 +1251,9 @@
       <c r="F42" s="4" t="n"/>
       <c r="G42" s="4" t="n"/>
       <c r="H42" s="4" t="n"/>
-    </row>
-    <row r="43" ht="16" customHeight="1">
+      <c r="I42" s="4" t="n"/>
+    </row>
+    <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
           <t>Action Release</t>
@@ -1251,8 +1266,9 @@
       <c r="F43" s="6" t="inlineStr"/>
       <c r="G43" s="6" t="inlineStr"/>
       <c r="H43" s="6" t="inlineStr"/>
-    </row>
-    <row r="44" ht="50" customHeight="1">
+      <c r="I43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44" ht="55" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
         <is>
           <t>Video</t>
@@ -1262,55 +1278,58 @@
       <c r="C44" s="6" t="inlineStr"/>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Creator video #2 — community lead POV</t>
+          <t>Creator video #2 - community lead POV</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr"/>
       <c r="F44" s="6" t="inlineStr"/>
       <c r="G44" s="6" t="inlineStr"/>
       <c r="H44" s="6" t="inlineStr"/>
-    </row>
-    <row r="45" ht="50" customHeight="1">
+      <c r="I44" s="4" t="inlineStr"/>
+    </row>
+    <row r="45" ht="55" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>X — Announcement</t>
-        </is>
-      </c>
-      <c r="B45" s="8" t="inlineStr">
-        <is>
-          <t>Campaign of the Week — spotlight (POST, recurring)</t>
+          <t>X - Announcement</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Campaign of the Week - spotlight (POST, recurring)</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr"/>
       <c r="D45" s="6" t="inlineStr"/>
       <c r="E45" s="6" t="inlineStr"/>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>Best campaigns so far — curated recap (POST)</t>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>Best campaigns so far - curated recap (POST)</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr"/>
       <c r="H45" s="6" t="inlineStr"/>
-    </row>
-    <row r="46" ht="50" customHeight="1">
+      <c r="I45" s="4" t="inlineStr"/>
+    </row>
+    <row r="46" ht="55" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>X — Sell to Projects</t>
+          <t>X - Sell to Projects</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr"/>
       <c r="C46" s="6" t="inlineStr"/>
       <c r="D46" s="6" t="inlineStr"/>
-      <c r="E46" s="11" t="inlineStr">
-        <is>
-          <t>Case study THREAD: first Verified Campaign — results, ROI, what they unlocked</t>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>Case study THREAD: first Verified Campaign - results, ROI, what they unlocked</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr"/>
       <c r="G46" s="6" t="inlineStr"/>
       <c r="H46" s="6" t="inlineStr"/>
-    </row>
-    <row r="47" ht="50" customHeight="1">
+      <c r="I46" s="4" t="inlineStr"/>
+    </row>
+    <row r="47" ht="55" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
         <is>
           <t>Article</t>
@@ -1319,7 +1338,7 @@
       <c r="B47" s="6" t="inlineStr"/>
       <c r="C47" s="6" t="inlineStr"/>
       <c r="D47" s="6" t="inlineStr"/>
-      <c r="E47" s="9" t="inlineStr">
+      <c r="E47" s="7" t="inlineStr">
         <is>
           <t>Case study: first Verified Campaign (ARTICLE)</t>
         </is>
@@ -1327,8 +1346,9 @@
       <c r="F47" s="6" t="inlineStr"/>
       <c r="G47" s="6" t="inlineStr"/>
       <c r="H47" s="6" t="inlineStr"/>
-    </row>
-    <row r="48" ht="16" customHeight="1">
+      <c r="I47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
           <t>X Space / Live</t>
@@ -1341,8 +1361,9 @@
       <c r="F48" s="6" t="inlineStr"/>
       <c r="G48" s="6" t="inlineStr"/>
       <c r="H48" s="6" t="inlineStr"/>
-    </row>
-    <row r="49" ht="16" customHeight="1">
+      <c r="I48" s="4" t="inlineStr"/>
+    </row>
+    <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
           <t>Creators &amp; Communities</t>
@@ -1355,8 +1376,9 @@
       <c r="F49" s="6" t="inlineStr"/>
       <c r="G49" s="6" t="inlineStr"/>
       <c r="H49" s="6" t="inlineStr"/>
-    </row>
-    <row r="50" ht="50" customHeight="1">
+      <c r="I49" s="4" t="inlineStr"/>
+    </row>
+    <row r="50" ht="55" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
         <is>
           <t>BD / Projects</t>
@@ -1373,8 +1395,9 @@
       <c r="F50" s="6" t="inlineStr"/>
       <c r="G50" s="6" t="inlineStr"/>
       <c r="H50" s="6" t="inlineStr"/>
-    </row>
-    <row r="51" ht="50" customHeight="1">
+      <c r="I50" s="4" t="inlineStr"/>
+    </row>
+    <row r="51" ht="55" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
         <is>
           <t>PR</t>
@@ -1391,8 +1414,9 @@
       <c r="F51" s="6" t="inlineStr"/>
       <c r="G51" s="6" t="inlineStr"/>
       <c r="H51" s="6" t="inlineStr"/>
-    </row>
-    <row r="52" ht="50" customHeight="1">
+      <c r="I51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52" ht="55" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
         <is>
           <t>Mailing</t>
@@ -1403,14 +1427,15 @@
       <c r="D52" s="6" t="inlineStr"/>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Case study to pipeline — 'this could be your launch'</t>
+          <t>Case study to pipeline - 'this could be your launch'</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr"/>
       <c r="G52" s="6" t="inlineStr"/>
       <c r="H52" s="6" t="inlineStr"/>
-    </row>
-    <row r="53" ht="50" customHeight="1">
+      <c r="I52" s="4" t="inlineStr"/>
+    </row>
+    <row r="53" ht="55" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
         <is>
           <t>KOL</t>
@@ -1427,11 +1452,12 @@
       <c r="F53" s="6" t="inlineStr"/>
       <c r="G53" s="6" t="inlineStr"/>
       <c r="H53" s="6" t="inlineStr"/>
+      <c r="I53" s="4" t="inlineStr"/>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Week of Aug 31 – Sep 06, 2026 (MOMENTUM — light week)</t>
+          <t>Week of Aug 31 - Sep 06, 2026 (MOMENTUM - light week)</t>
         </is>
       </c>
       <c r="B55" s="4" t="n"/>
@@ -1441,8 +1467,9 @@
       <c r="F55" s="4" t="n"/>
       <c r="G55" s="4" t="n"/>
       <c r="H55" s="4" t="n"/>
-    </row>
-    <row r="56" ht="16" customHeight="1">
+      <c r="I55" s="4" t="n"/>
+    </row>
+    <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
           <t>Action Release</t>
@@ -1455,8 +1482,9 @@
       <c r="F56" s="6" t="inlineStr"/>
       <c r="G56" s="6" t="inlineStr"/>
       <c r="H56" s="6" t="inlineStr"/>
-    </row>
-    <row r="57" ht="50" customHeight="1">
+      <c r="I56" s="4" t="inlineStr"/>
+    </row>
+    <row r="57" ht="55" customHeight="1">
       <c r="A57" s="5" t="inlineStr">
         <is>
           <t>Video</t>
@@ -1473,16 +1501,17 @@
       <c r="F57" s="6" t="inlineStr"/>
       <c r="G57" s="6" t="inlineStr"/>
       <c r="H57" s="6" t="inlineStr"/>
-    </row>
-    <row r="58" ht="50" customHeight="1">
+      <c r="I57" s="4" t="inlineStr"/>
+    </row>
+    <row r="58" ht="55" customHeight="1">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>X — Announcement</t>
-        </is>
-      </c>
-      <c r="B58" s="8" t="inlineStr">
-        <is>
-          <t>Numbers post — month in review (show numbers) + Campaign of the Week</t>
+          <t>X - Announcement</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Numbers post - month in review (show numbers) + Campaign of the Week</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr"/>
@@ -1490,31 +1519,33 @@
       <c r="E58" s="6" t="inlineStr"/>
       <c r="F58" s="6" t="inlineStr"/>
       <c r="G58" s="6" t="inlineStr"/>
-      <c r="H58" s="8" t="inlineStr">
-        <is>
-          <t>What's next — roadmap tease (POST)</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="50" customHeight="1">
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>What's next - roadmap tease (POST)</t>
+        </is>
+      </c>
+      <c r="I58" s="4" t="inlineStr"/>
+    </row>
+    <row r="59" ht="55" customHeight="1">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>X — Sell to Projects</t>
+          <t>X - Sell to Projects</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr"/>
       <c r="C59" s="6" t="inlineStr"/>
       <c r="D59" s="6" t="inlineStr"/>
       <c r="E59" s="6" t="inlineStr"/>
-      <c r="F59" s="11" t="inlineStr">
+      <c r="F59" s="7" t="inlineStr">
         <is>
           <t>Open call: September cohort for Network &amp; Verified Campaigns (POST)</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr"/>
       <c r="H59" s="6" t="inlineStr"/>
-    </row>
-    <row r="60" ht="16" customHeight="1">
+      <c r="I59" s="4" t="inlineStr"/>
+    </row>
+    <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
           <t>Article</t>
@@ -1527,8 +1558,9 @@
       <c r="F60" s="6" t="inlineStr"/>
       <c r="G60" s="6" t="inlineStr"/>
       <c r="H60" s="6" t="inlineStr"/>
-    </row>
-    <row r="61" ht="16" customHeight="1">
+      <c r="I60" s="4" t="inlineStr"/>
+    </row>
+    <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
           <t>X Space / Live</t>
@@ -1541,8 +1573,9 @@
       <c r="F61" s="6" t="inlineStr"/>
       <c r="G61" s="6" t="inlineStr"/>
       <c r="H61" s="6" t="inlineStr"/>
-    </row>
-    <row r="62" ht="16" customHeight="1">
+      <c r="I61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
           <t>Creators &amp; Communities</t>
@@ -1555,8 +1588,9 @@
       <c r="F62" s="6" t="inlineStr"/>
       <c r="G62" s="6" t="inlineStr"/>
       <c r="H62" s="6" t="inlineStr"/>
-    </row>
-    <row r="63" ht="16" customHeight="1">
+      <c r="I62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
           <t>BD / Projects</t>
@@ -1569,8 +1603,9 @@
       <c r="F63" s="6" t="inlineStr"/>
       <c r="G63" s="6" t="inlineStr"/>
       <c r="H63" s="6" t="inlineStr"/>
-    </row>
-    <row r="64" ht="16" customHeight="1">
+      <c r="I63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
           <t>PR</t>
@@ -1583,8 +1618,9 @@
       <c r="F64" s="6" t="inlineStr"/>
       <c r="G64" s="6" t="inlineStr"/>
       <c r="H64" s="6" t="inlineStr"/>
-    </row>
-    <row r="65" ht="50" customHeight="1">
+      <c r="I64" s="4" t="inlineStr"/>
+    </row>
+    <row r="65" ht="55" customHeight="1">
       <c r="A65" s="5" t="inlineStr">
         <is>
           <t>Mailing</t>
@@ -1601,8 +1637,9 @@
       </c>
       <c r="G65" s="6" t="inlineStr"/>
       <c r="H65" s="6" t="inlineStr"/>
-    </row>
-    <row r="66" ht="16" customHeight="1">
+      <c r="I65" s="4" t="inlineStr"/>
+    </row>
+    <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
           <t>KOL</t>
@@ -1615,122 +1652,123 @@
       <c r="F66" s="6" t="inlineStr"/>
       <c r="G66" s="6" t="inlineStr"/>
       <c r="H66" s="6" t="inlineStr"/>
+      <c r="I66" s="4" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="12" t="inlineStr">
+      <c r="A68" s="9" t="inlineStr">
         <is>
           <t>How to read this calendar</t>
         </is>
       </c>
-      <c r="B68" s="13" t="inlineStr"/>
-    </row>
-    <row r="69" ht="30" customHeight="1">
-      <c r="A69" s="12" t="inlineStr">
+      <c r="B68" s="10" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="inlineStr">
         <is>
           <t>Logic of the month</t>
         </is>
       </c>
-      <c r="B69" s="13" t="inlineStr">
-        <is>
-          <t>W1 narrative + teaser -&gt; W2 launch (Demo Video + Verified/Network threads + call for projects) -&gt; W3 sell to projects + creators (live demo + Space ~1 week after launch) -&gt; W4 social proof + PR (~2 weeks after launch, with real numbers) -&gt; W5 momentum, light.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="30" customHeight="1">
-      <c r="A70" s="12" t="inlineStr">
+      <c r="B69" s="10" t="inlineStr">
+        <is>
+          <t>W1 narrative + teaser, W2 launch (Demo Video + Verified/Network threads + call for projects), W3 sell to projects + creators (live demo + Space one week after launch), W4 social proof + PR (two weeks after launch, with real numbers), W5 momentum, light.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="9" t="inlineStr">
         <is>
           <t>X-first</t>
         </is>
       </c>
-      <c r="B70" s="13" t="inlineStr">
-        <is>
-          <t>Everything runs on X (posts, threads, Spaces, live demo). No Discord/Telegram. 'X — Sell to Projects' (pink) is content aimed directly at projects: Verified/Network pitches, call for projects, case study ROI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="30" customHeight="1">
-      <c r="A71" s="12" t="inlineStr">
+      <c r="B70" s="10" t="inlineStr">
+        <is>
+          <t>Everything runs on X (posts, threads, Spaces, live demo). No Discord/Telegram. 'X - Sell to Projects' is content aimed directly at projects: Verified/Network pitches, call for projects, case study ROI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="9" t="inlineStr">
         <is>
           <t>Mailing</t>
         </is>
       </c>
-      <c r="B71" s="13" t="inlineStr">
+      <c r="B71" s="10" t="inlineStr">
         <is>
           <t>Only for key articles and important calls to the project pipeline: launch, Verified one-pager, 'Why Network Campaigns', case study, monthly recap + cohort call.</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="30" customHeight="1">
-      <c r="A72" s="12" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="9" t="inlineStr">
         <is>
           <t>Reusable assets</t>
         </is>
       </c>
-      <c r="B72" s="13" t="inlineStr">
+      <c r="B72" s="10" t="inlineStr">
         <is>
           <t>Demo Video (+ cutdowns), Verified one-pager, Verified vs Network visual, use-cases &amp; playbook articles, creator videos and the case study all double as sales material for pitching projects.</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="30" customHeight="1">
-      <c r="A73" s="12" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="9" t="inlineStr">
         <is>
           <t>Verified Campaigns</t>
         </is>
       </c>
-      <c r="B73" s="13" t="inlineStr">
+      <c r="B73" s="10" t="inlineStr">
         <is>
           <t>Verification filter + 1,500$. They get: protocol visibility/positioning, marketing service pack from Rally socials (articles, videos), and unlock of community &amp; elite creators features (ambassadors + campaign management in Rally).</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="30" customHeight="1">
-      <c r="A74" s="12" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="9" t="inlineStr">
         <is>
           <t>Network Campaigns</t>
         </is>
       </c>
-      <c r="B74" s="13" t="inlineStr">
-        <is>
-          <t>Permissionless — anyone can create a campaign. Rewards only in USDC or RLPs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="30" customHeight="1">
-      <c r="A75" s="12" t="inlineStr">
+      <c r="B74" s="10" t="inlineStr">
+        <is>
+          <t>Permissionless - anyone can create a campaign. Rewards only in USDC or RLPs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="9" t="inlineStr">
         <is>
           <t>Creator videos</t>
         </is>
       </c>
-      <c r="B75" s="13" t="inlineStr">
+      <c r="B75" s="10" t="inlineStr">
         <is>
           <t>3 short testimonial videos (briefed W1, recorded W2-W3, published W3-W5): creator experience, community lead POV, month recap.</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="12" t="inlineStr"/>
-      <c r="B76" s="13" t="inlineStr"/>
-    </row>
-    <row r="77" ht="30" customHeight="1">
-      <c r="A77" s="12" t="inlineStr">
+      <c r="A76" s="9" t="inlineStr"/>
+      <c r="B76" s="10" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="9" t="inlineStr">
         <is>
           <t>Internal Campaigns doc</t>
         </is>
       </c>
-      <c r="B77" s="13" t="inlineStr">
+      <c r="B77" s="10" t="inlineStr">
         <is>
           <t>https://docs.google.com/document/d/13DhJE-HBozbZijic54TgX2L6m8FPw_oHp-_uZ1aOzuQ/edit?usp=sharing</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="30" customHeight="1">
-      <c r="A78" s="12" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="9" t="inlineStr">
         <is>
           <t>Rally Tracker</t>
         </is>
       </c>
-      <c r="B78" s="13" t="inlineStr">
+      <c r="B78" s="10" t="inlineStr">
         <is>
           <t>https://rally-tracker-ten.vercel.app/</t>
         </is>
@@ -1748,11 +1786,11 @@
     <mergeCell ref="B75:H75"/>
     <mergeCell ref="B73:H73"/>
     <mergeCell ref="B77:H77"/>
+    <mergeCell ref="A1:I1"/>
     <mergeCell ref="A42:H42"/>
     <mergeCell ref="B69:H69"/>
     <mergeCell ref="B70:H70"/>
     <mergeCell ref="B78:H78"/>
-    <mergeCell ref="A1:H1"/>
     <mergeCell ref="B72:H72"/>
     <mergeCell ref="B76:H76"/>
   </mergeCells>

</xml_diff>